<commit_message>
Butcher cannon range 48"; Thunderblast Cannon range back to 72"
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqADDPrpWypr4ibm6XufKK
</commit_message>
<xml_diff>
--- a/homebrew/reports/Weapon-Lists.xlsx
+++ b/homebrew/reports/Weapon-Lists.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Melee Weapons'!$A$1:$J$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Grenades'!$A$1:$J$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ranged Weapons'!$A$1:$J$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ranged Weapons'!$A$1:$J$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6794,7 +6794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>36"</t>
+          <t>48"</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -7056,27 +7056,23 @@
           <t>Heavy 3, Rending (6+), Twin-linked</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>2 different profiles</t>
-        </is>
-      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr"/>
+          <t>2022 - Legiones Astartes, 2022 - Mech Library</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>2022 - BG - Blackshields, 2022 - Mechanicum</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Butcher cannon</t>
+          <t>Chem Cannon</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -7086,49 +7082,37 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>48"</t>
+          <t>Template</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Heavy 3, Rending (6+), Twin-linked</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>2 different profiles</t>
-        </is>
-      </c>
+          <t>Heavy 1, Breaching (5+), Fleshbane</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>2022 - Mech Library</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>2022 - BG - Blackshields, 2022 - Legiones Astartes, 2022 - Mechanicum</t>
-        </is>
-      </c>
+          <t>2022 - LI - Solar Auxilia, Homebrew - Astra Militarum</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Chem Cannon</t>
+          <t>Cyclone Missile Launcher -  Flak</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -7138,29 +7122,29 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Template</t>
+          <t>48"</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Breaching (5+), Fleshbane</t>
+          <t>Heavy 2, Skyfire, Twin-linked</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia, Homebrew - Astra Militarum</t>
+          <t>2022 - Horus Heresy, 2022 - LI - Solar Auxilia</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr"/>
@@ -7168,7 +7152,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Cyclone Missile Launcher -  Flak</t>
+          <t>Cyclone Missile Launcher -  Krak</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -7183,7 +7167,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -7193,14 +7177,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Heavy 2, Skyfire, Twin-linked</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr"/>
+          <t>Heavy 2, Twin-linked</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>To verify</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>2 different profiles (wording/order only)</t>
+        </is>
+      </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, 2022 - LI - Solar Auxilia</t>
+          <t>2022 - LI - Solar Auxilia</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
@@ -7233,7 +7225,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Heavy 2, Twin-linked</t>
+          <t>Heavy 2. Twin-linked</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -7248,15 +7240,19 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Legiones Astartes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Cyclone Missile Launcher -  Krak</t>
+          <t>Disintegrator</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -7266,49 +7262,41 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>48"</t>
+          <t>24"</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Heavy 2. Twin-linked</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>2 different profiles (wording/order only)</t>
-        </is>
-      </c>
+          <t>Rapid Fire, Instant Death, Gets Hot</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy</t>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
+          <t>2022 - LI - Sisters Of Silence, 2022 - Legiones Astartes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Disintegrator</t>
+          <t>Disintegrator Cannon</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -7318,12 +7306,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>24"</t>
+          <t>36"</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -7333,26 +7321,22 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Rapid Fire, Instant Death, Gets Hot</t>
+          <t>Heavy 2, Rending (5+), Sunder</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LI - Sisters Of Silence, 2022 - Legiones Astartes</t>
-        </is>
-      </c>
+          <t>2022 - Legiones Astartes, Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Drukhari)</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Disintegrator Cannon</t>
+          <t>Disintegrator Pistol</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -7362,12 +7346,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>36"</t>
+          <t>12"</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -7377,22 +7361,26 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Heavy 2, Rending (5+), Sunder</t>
+          <t>Pistol 1, Instant Death, Gets Hot</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes, Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Drukhari)</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - Death Guard, 2022 - LI - Sisters Of Silence, 2022 - Legiones Astartes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Disintegrator Pistol</t>
+          <t>Eradicator Nova Cannon</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -7402,41 +7390,37 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>12"</t>
+          <t>36"</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Pistol 1, Instant Death, Gets Hot</t>
+          <t>Heavy 1, Large Blast (5"), Ignores Cover</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - Death Guard, 2022 - LI - Sisters Of Silence, 2022 - Legiones Astartes</t>
-        </is>
-      </c>
+          <t>2022 - LI - Solar Auxilia, Homebrew - Astra Militarum</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Eradicator Nova Cannon</t>
+          <t>Extinctor power claw and a manipulator arm</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -7444,31 +7428,23 @@
           <t>Ranged</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>36"</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Heavy 1, Large Blast (5"), Ignores Cover</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="4" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>To verify</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>blank characteristic</t>
+        </is>
+      </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia, Homebrew - Astra Militarum</t>
+          <t>2022 - LA - Dark Angels</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
@@ -7476,7 +7452,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Extinctor power claw and a manipulator arm</t>
+          <t>Eyrine Needle Pistol</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -7484,23 +7460,31 @@
           <t>Ranged</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr"/>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>blank characteristic</t>
-        </is>
-      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>12"</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Pistol 2, Poisoned (3+), Pinning, Master-crafted</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Dark Angels</t>
+          <t>2022 - LI - Sisters Of Silence</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr"/>
@@ -7508,7 +7492,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Eyrine Needle Pistol</t>
+          <t>Fusion pistol</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -7518,29 +7502,29 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>12"</t>
+          <t>8"</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Pistol 2, Poisoned (3+), Pinning, Master-crafted</t>
+          <t>Pistol 1, Armourbane (Melta)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Sisters Of Silence</t>
+          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani), Homebrew - Aeldari (Rillietann), Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
@@ -7548,7 +7532,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Fusion pistol</t>
+          <t>Gravis Melta Cannon</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -7558,7 +7542,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>8"</t>
+          <t>24"</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -7573,22 +7557,26 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Pistol 1, Armourbane (Melta)</t>
+          <t>Heavy 2, Armourbane (Melta), Twin-linked</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani), Homebrew - Aeldari (Rillietann), Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - Thousand Sons, 2022 - LA - Word Bearers, 2022 - LI - Custodes, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Gravis Melta Cannon</t>
+          <t>Gravis Multi-Laser</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -7598,41 +7586,41 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>24"</t>
+          <t>36"</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Heavy 2, Armourbane (Melta), Twin-linked</t>
+          <t>Heavy 6, Twin-linked</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+          <t>2022 - Horus Heresy</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Thousand Sons, 2022 - LA - Word Bearers, 2022 - LI - Custodes, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes</t>
+          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, Homebrew - Traders Militant</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Gravis Multi-Laser</t>
+          <t>Graviton Gun</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -7642,41 +7630,41 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>36"</t>
+          <t>18"</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>†</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Heavy 6, Twin-linked</t>
+          <t>Heavy 1, Blast (3"), Concussive (1), Graviton Pulse, Haywire</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy</t>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, Homebrew - Traders Militant</t>
+          <t>2022 - LA - Dark Angels, 2022 - LA - Iron Hands, 2022 - LA - Thousand Sons, 2022 - LA - Ultramarines, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mech Library, 2022 - Mechanicum</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Graviton Gun</t>
+          <t>Graviton Imploder</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -7696,31 +7684,31 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Blast (3"), Concussive (1), Graviton Pulse, Haywire</t>
+          <t>Heavy 2, Concussive (1), Graviton Pulse, Haywire</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+          <t>2022 - Mech Library, Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Dark Angels, 2022 - LA - Iron Hands, 2022 - LA - Thousand Sons, 2022 - LA - Ultramarines, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mech Library, 2022 - Mechanicum</t>
+          <t>2022 - Mechanicum</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Graviton Imploder</t>
+          <t>Havoc Launcher</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -7730,41 +7718,41 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>18"</t>
+          <t>48"</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>†</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Heavy 2, Concussive (1), Graviton Pulse, Haywire</t>
+          <t>Heavy 1, Blast (3"), Twin-linked</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr"/>
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2022 - Mech Library, Homebrew - Traders Militant</t>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>2022 - Mechanicum</t>
+          <t>2022 - Imperialis Militia, 2022 - LA - Thousand Sons, 2022 - LI - Custodes, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Havoc Launcher</t>
+          <t>Haywire cannon</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -7774,41 +7762,37 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>48"</t>
+          <t>36"</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Blast (3"), Twin-linked</t>
+          <t>Assault 3, Haywire</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr"/>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia, 2022 - LA - Thousand Sons, 2022 - LI - Custodes, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum</t>
-        </is>
-      </c>
+          <t>Homebrew - Aeldari (Drukhari), Homebrew - Aeldari (Rillietann)</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Haywire cannon</t>
+          <t>Heavy Frag Rocket</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -7828,27 +7812,31 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Assault 3, Haywire</t>
+          <t>Heavy 1, Blast (3"), Pinning, One Use</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Drukhari), Homebrew - Aeldari (Rillietann)</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Heavy Frag Rocket</t>
+          <t>Heavy Krak Rocket</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -7863,17 +7851,17 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Blast (3"), Pinning, One Use</t>
+          <t>Heavy 1, One Use</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr"/>
@@ -7892,7 +7880,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Heavy Krak Rocket</t>
+          <t>Heavy Lascannon</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -7902,29 +7890,29 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>36"</t>
+          <t>48"</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, One Use</t>
+          <t>Heavy 1, Sunder</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr"/>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy</t>
+          <t>2022 - Horus Heresy, Homebrew - Astra Militarum</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -7936,7 +7924,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Heavy Lascannon</t>
+          <t>Hellstrike Missile</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -7946,12 +7934,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>48"</t>
+          <t>72"</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -7961,7 +7949,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Sunder</t>
+          <t>Heavy 1, Sunder, One Shot</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr"/>
@@ -7973,14 +7961,14 @@
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia</t>
+          <t>2022 - LA - Imperial Fists, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Hellstrike Missile</t>
+          <t>Hot-Shot Laspistol</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -7990,41 +7978,37 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>72"</t>
+          <t>9"</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Sunder, One Shot</t>
+          <t>Pistol 1</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr"/>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Astra Militarum</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - Imperial Fists, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes</t>
-        </is>
-      </c>
+          <t>2022 - LI - Solar Auxilia, Homebrew - Astra Militarum, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Hot-Shot Laspistol</t>
+          <t>Hot-Shot Volley Gun</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -8034,22 +8018,22 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>9"</t>
+          <t>24"</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Pistol 1</t>
+          <t>Heavy 4</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr"/>
@@ -8064,7 +8048,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Hot-Shot Volley Gun</t>
+          <t>Hyperios Missile Launcher</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -8074,12 +8058,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>24"</t>
+          <t>48"</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -8089,22 +8073,26 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Heavy 4</t>
+          <t>Heavy 3, Skyfire</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr"/>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia, Homebrew - Astra Militarum, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, 2022 - Legiones Astartes, 2022 - Mechanicum</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LI - Solar Auxilia</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Hyperios Missile Launcher</t>
+          <t>Impaler harpoon</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -8114,41 +8102,41 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>48"</t>
+          <t>12"</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Heavy 3, Skyfire</t>
+          <t>Heavy 1, Impale</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr"/>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, 2022 - Legiones Astartes, 2022 - Mechanicum</t>
+          <t>2022 - Legiones Astartes, 2022 - Mech Library</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia</t>
+          <t>2022 - Mechanicum</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Impaler harpoon</t>
+          <t>Inferno Cannon</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -8158,7 +8146,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>12"</t>
+          <t>Hellstorm</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -8168,31 +8156,27 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Impale</t>
+          <t>Ordnance 1, Torrent (9"), Breaching (6+), Concussive (1)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes, 2022 - Mech Library</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Mechanicum</t>
-        </is>
-      </c>
+          <t>2022 - LI - Solar Auxilia, Homebrew - Astra Militarum</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Inferno Cannon</t>
+          <t>Irad-Cleanser</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -8202,37 +8186,41 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Hellstorm</t>
+          <t>Template</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Ordnance 1, Torrent (9"), Breaching (6+), Concussive (1)</t>
+          <t>Assault 1, Fleshbane, Rad-phage</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr"/>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia, Homebrew - Astra Militarum</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - Dark Angels, 2022 - Mech Library, 2022 - Mechanicum</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Irad-Cleanser</t>
+          <t>Lucifex</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -8242,7 +8230,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Template</t>
+          <t>8"</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -8257,110 +8245,110 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Assault 1, Fleshbane, Rad-phage</t>
+          <t>Pistol 1, Fleshbane, Rad-phage</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr"/>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+          <t>2022 - Mech Library, Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Dark Angels, 2022 - Mech Library, 2022 - Mechanicum</t>
+          <t>2022 - Mechanicum</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>Lucifex</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Medusa Mortar</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Ranged</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>8"</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>Pistol 1, Fleshbane, Rad-phage</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Mech Library, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Mechanicum</t>
-        </is>
-      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>36"</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Ordnance 1, Large Blast (5"), Barrage, Shred, Rupture (6+)</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr"/>
+      <c r="H35" s="7" t="inlineStr"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Artillery Weapons)</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Medusa Mortar</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Ranged</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>36"</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>Ordnance 1, Large Blast (5"), Barrage, Shred, Rupture (6+)</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr"/>
-      <c r="H36" s="7" t="inlineStr"/>
-      <c r="I36" s="7" t="inlineStr">
-        <is>
-          <t>Master list (Artillery Weapons)</t>
-        </is>
-      </c>
-      <c r="J36" s="7" t="inlineStr"/>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="4" t="inlineStr"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Horus Heresy, 2022 - Imperialis Militia</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Medusa Mortar</t>
+          <t>Melta Cannon</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -8370,41 +8358,41 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>36"</t>
+          <t>60"</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Ordnance 1, Large Blast (5"), Barrage, Shred, Rupture (6+)</t>
+          <t>Heavy 1, Massive Blast (7"), Armourbane (Melta)</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, 2022 - Imperialis Militia</t>
+          <t>2022 - Horus Heresy, Homebrew - Astra Militarum</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum</t>
+          <t>2022 - LI - Solar Auxilia, 2022 - Mech Library</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Melta Cannon</t>
+          <t>Melta Lance</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -8414,12 +8402,12 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>60"</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -8429,26 +8417,30 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Massive Blast (7"), Armourbane (Melta)</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="4" t="inlineStr"/>
+          <t>Heavy 1, Armourbane (Ranged)</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>To verify</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>2 different profiles; differs from master list</t>
+        </is>
+      </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Astra Militarum</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LI - Solar Auxilia, 2022 - Mech Library</t>
-        </is>
-      </c>
+          <t>2022 - LI - Solar Auxilia</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Melta Lance</t>
+          <t>Mortar</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -8458,37 +8450,29 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>48"</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Armourbane (Ranged)</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H39" s="5" t="inlineStr">
-        <is>
-          <t>2 different profiles; differs from master list</t>
-        </is>
-      </c>
+          <t>Heavy 1, Blast (3"), Barrage, Pinning</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia</t>
+          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, Homebrew - Astra Militarum</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr"/>
@@ -8496,7 +8480,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Mortar</t>
+          <t>Multiple Rocket Pod</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -8506,7 +8490,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>48"</t>
+          <t>24"</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -8521,14 +8505,14 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Blast (3"), Barrage, Pinning</t>
+          <t>Heavy 1, Large Blast (5"), Pinning</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, Homebrew - Astra Militarum</t>
+          <t>2022 - LI - Solar Auxilia, Homebrew - Astra Militarum</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr"/>
@@ -8536,7 +8520,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Multiple Rocket Pod</t>
+          <t>Needle Pistol</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -8546,37 +8530,41 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>24"</t>
+          <t>12"</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Large Blast (5"), Pinning</t>
+          <t>Pistol 2, Poisoned (3+), Pinning</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia, Homebrew - Astra Militarum</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, 2022 - LA - Dark Angels</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia, 2022 - LA - Alpha Legion, 2022 - LI - Assassins, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, Homebrew - Traders Militant</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Needle Pistol</t>
+          <t>Neuro disruptor</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -8591,36 +8579,32 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Pistol 2, Poisoned (3+), Pinning</t>
+          <t>Pistol 1, Fleshbane</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, 2022 - LA - Dark Angels</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia, 2022 - LA - Alpha Legion, 2022 - LI - Assassins, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, Homebrew - Traders Militant</t>
-        </is>
-      </c>
+          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Rillietann), Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Neuro disruptor</t>
+          <t>Omega Pattern Plasma Blastgun</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -8630,29 +8614,37 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>12"</t>
+          <t>36"</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Pistol 1, Fleshbane</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
+          <t>Ordnance 1, Gets Hot, Massive Blast (7"), Rending (4+)</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>To verify</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>2 different profiles</t>
+        </is>
+      </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Rillietann), Homebrew - Traders Militant</t>
+          <t>2022 - Legiones Astartes</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr"/>
@@ -8670,7 +8662,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>36"</t>
+          <t>48"</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -8700,7 +8692,7 @@
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
+          <t>2022 - LI - Solar Auxilia</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr"/>
@@ -8708,7 +8700,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Omega Pattern Plasma Blastgun</t>
+          <t>Particle Shredder</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -8718,37 +8710,29 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>48"</t>
+          <t>8"</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Ordnance 1, Gets Hot, Massive Blast (7"), Rending (4+)</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H45" s="5" t="inlineStr">
-        <is>
-          <t>2 different profiles</t>
-        </is>
-      </c>
+          <t>Assault 3, Shred</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia</t>
+          <t>2022 - Legiones Astartes</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr"/>
@@ -8756,7 +8740,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Particle Shredder</t>
+          <t>Photon Thruster</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -8766,7 +8750,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>8"</t>
+          <t>24"</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -8776,27 +8760,31 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Assault 3, Shred</t>
+          <t>Assault 2, Blind, Lance, Gets Hot</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr"/>
       <c r="H46" s="4" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="inlineStr"/>
+          <t>2022 - Mech Library, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Mechanicum</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Photon Thruster</t>
+          <t>Ranger long rifle</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -8806,41 +8794,37 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>24"</t>
+          <t>48"</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Assault 2, Blind, Lance, Gets Hot</t>
+          <t>Heavy 1, Pinning, Rending (5+), Sniper</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr"/>
       <c r="H47" s="4" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>2022 - Mech Library, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Mechanicum</t>
-        </is>
-      </c>
+          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani), Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Ranger long rifle</t>
+          <t>Ripper Gun</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -8850,7 +8834,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>48"</t>
+          <t>12"</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -8860,27 +8844,39 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Pinning, Rending (5+), Sniper</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr"/>
-      <c r="H48" s="4" t="inlineStr"/>
+          <t>Assault 5</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>To verify</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>differs from master list</t>
+        </is>
+      </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani), Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J48" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, Homebrew - Astra Militarum</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Ripper Gun</t>
+          <t>Scorpion cannon</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -8890,49 +8886,41 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>12"</t>
+          <t>36"</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Assault 5</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>differs from master list</t>
-        </is>
-      </c>
+          <t>Assault 9, Pinning, Shred</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr"/>
+      <c r="H49" s="4" t="inlineStr"/>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Astra Militarum</t>
+          <t>2022 - Legiones Astartes, 2022 - Mech Library</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia</t>
+          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, 2022 - Mechanicum</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Scorpion cannon</t>
+          <t>Shotgun</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -8942,41 +8930,41 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>36"</t>
+          <t>12"</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Assault 9, Pinning, Shred</t>
+          <t>Assault 2, Concussive (1)</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr"/>
       <c r="H50" s="4" t="inlineStr"/>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes, 2022 - Mech Library</t>
+          <t>2022 - Horus Heresy, Homebrew - Astra Militarum</t>
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, 2022 - Mechanicum</t>
+          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, Homebrew - Traders Militant</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Shotgun</t>
+          <t>Shuriken catapult</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -8986,41 +8974,37 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>12"</t>
+          <t>18"</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Assault 2, Concussive (1)</t>
+          <t>Assault 2, Breaching (6+)</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr"/>
       <c r="H51" s="4" t="inlineStr"/>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Astra Militarum</t>
-        </is>
-      </c>
-      <c r="J51" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, Homebrew - Traders Militant</t>
-        </is>
-      </c>
+          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani), Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Shuriken catapult</t>
+          <t>Shuriken pistol</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -9030,7 +9014,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>18"</t>
+          <t>12"</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -9045,14 +9029,14 @@
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Assault 2, Breaching (6+)</t>
+          <t>Pistol 1, Breaching (6+)</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr"/>
       <c r="H52" s="4" t="inlineStr"/>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani), Homebrew - Traders Militant</t>
+          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani), Homebrew - Aeldari (Rillietann), Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr"/>
@@ -9060,7 +9044,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Shuriken pistol</t>
+          <t>Singing spear (ranged)</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -9075,24 +9059,32 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Pistol 1, Breaching (6+)</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr"/>
-      <c r="H53" s="4" t="inlineStr"/>
+          <t>Assault 1</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>To verify</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>2 different profiles</t>
+        </is>
+      </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani), Homebrew - Aeldari (Rillietann), Homebrew - Traders Militant</t>
+          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani)</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr"/>
@@ -9120,12 +9112,12 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Assault 1</t>
+          <t>Assault 1, Soul Tear</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
@@ -9148,7 +9140,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Singing spear (ranged)</t>
+          <t>Sniper Rifle</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -9158,45 +9150,41 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>12"</t>
+          <t>72"</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>Assault 1, Soul Tear</t>
-        </is>
-      </c>
-      <c r="G55" s="3" t="inlineStr">
-        <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H55" s="5" t="inlineStr">
-        <is>
-          <t>2 different profiles</t>
-        </is>
-      </c>
+          <t>Heavy 1, Rending (5+), Sniper, Pinning</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr"/>
+      <c r="H55" s="4" t="inlineStr"/>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani)</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, Homebrew - Astra Militarum</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia, 2022 - Legiones Astartes</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Sniper Rifle</t>
+          <t>Sonic Lance</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -9206,41 +9194,41 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>72"</t>
+          <t>Template</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Rending (5+), Sniper, Pinning</t>
+          <t>Assault 1, Breaching (6+), Pinning</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr"/>
       <c r="H56" s="4" t="inlineStr"/>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Astra Militarum</t>
+          <t>2022 - Legiones Astartes</t>
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia, 2022 - Legiones Astartes</t>
+          <t>2022 - LA - Emperor's Children</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Sonic Lance</t>
+          <t>Soulburner petard</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -9250,41 +9238,41 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Template</t>
+          <t>24"</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Assault 1, Breaching (6+), Pinning</t>
+          <t>Heavy 1, Blast (3"), Breaching (5+), Fleshbane</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr"/>
       <c r="H57" s="4" t="inlineStr"/>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
+          <t>2022 - Legiones Astartes, 2022 - Mech Library</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Emperor's Children</t>
+          <t>2022 - BG - Blackshields, 2022 - Mechanicum</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Soulburner petard</t>
+          <t>The Devil's Due</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -9294,125 +9282,125 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>24"</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Heavy 1, Blast (3"), Breaching (5+), Fleshbane</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr"/>
+          <t>Unwieldy (3), The Devil's Due, Murderous Strike (6+), Master-crafted</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
       <c r="H58" s="4" t="inlineStr"/>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes, 2022 - Mech Library</t>
-        </is>
-      </c>
-      <c r="J58" s="4" t="inlineStr">
-        <is>
-          <t>2022 - BG - Blackshields, 2022 - Mechanicum</t>
-        </is>
-      </c>
+          <t>2022 - LA - Night Lords</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>The Devil's Due</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Thunderblast Cannon</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>Ranged</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>+2</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>Unwieldy (3), The Devil's Due, Murderous Strike (6+), Master-crafted</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
-      <c r="H59" s="4" t="inlineStr"/>
-      <c r="I59" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - Night Lords</t>
-        </is>
-      </c>
-      <c r="J59" s="4" t="inlineStr"/>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>72"</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>Ordnance 1, Large Blast (5"), Rupture (5+), Pinning</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr"/>
+      <c r="H59" s="7" t="inlineStr"/>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Artillery Weapons)</t>
+        </is>
+      </c>
+      <c r="J59" s="7" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>Thunderblast Cannon</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>Ranged</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
-        <is>
-          <t>36"</t>
-        </is>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>72"</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="E60" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F60" s="7" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr">
         <is>
           <t>Ordnance 1, Large Blast (5"), Rupture (5+), Pinning</t>
         </is>
       </c>
-      <c r="G60" s="6" t="inlineStr"/>
-      <c r="H60" s="7" t="inlineStr"/>
-      <c r="I60" s="7" t="inlineStr">
-        <is>
-          <t>Master list (Artillery Weapons)</t>
-        </is>
-      </c>
-      <c r="J60" s="7" t="inlineStr"/>
+      <c r="G60" s="3" t="inlineStr"/>
+      <c r="H60" s="4" t="inlineStr"/>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Horus Heresy</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Thunderblast Cannon</t>
+          <t>Thunderstub</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -9422,12 +9410,12 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>36"</t>
+          <t>6"</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
@@ -9437,7 +9425,7 @@
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Ordnance 1, Large Blast (5"), Rupture (5+), Pinning</t>
+          <t>Pistol 1, Brutal (2), Concussive (1)</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr"/>
@@ -9456,7 +9444,7 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Thunderstub</t>
+          <t>Volkite Dual-Culverin</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -9466,7 +9454,7 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>6"</t>
+          <t>45"</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -9476,80 +9464,36 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Pistol 1, Brutal (2), Concussive (1)</t>
+          <t>Heavy 6, Deflagrate, Twin-linked</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr"/>
       <c r="H62" s="4" t="inlineStr"/>
       <c r="I62" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy</t>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J62" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>Volkite Dual-Culverin</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>Ranged</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>45"</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="inlineStr">
-        <is>
-          <t>Heavy 6, Deflagrate, Twin-linked</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="inlineStr"/>
-      <c r="H63" s="4" t="inlineStr"/>
-      <c r="I63" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J63" s="4" t="inlineStr">
-        <is>
           <t>2022 - LA - Thousand Sons, 2022 - LI - Custodes, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>Rows shaded blue are the master weapon list (homebrew/source/additional-weapons.md); other rows are catalogue/gst profiles. 'Defined in' is the file holding the profile; 'Used by' is catalogues linking to it.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J63"/>
+  <autoFilter ref="A1:J62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Power Pack wargear and Power Pack weapons to the game system
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqADDPrpWypr4ibm6XufKK
</commit_message>
<xml_diff>
--- a/homebrew/reports/Weapon-Lists.xlsx
+++ b/homebrew/reports/Weapon-Lists.xlsx
@@ -12,9 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ranged Weapons" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Melee Weapons'!$A$1:$J$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Melee Weapons'!$A$1:$J$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Grenades'!$A$1:$J$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ranged Weapons'!$A$1:$J$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ranged Weapons'!$A$1:$J$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J97"/>
+  <dimension ref="A1:J103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1194,53 +1194,49 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Corposant Stave</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>+1</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Circular Stone Saw</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Melee, Haywire, Two-handed</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia, 2022 - Legiones Astartes, 2022 - Mechanicum, 2022 - Titan Legions</t>
-        </is>
-      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Melee, Shred</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr"/>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Power Pack Weapons)</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Crushing fists</t>
+          <t>Circular Stone Saw</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1255,7 +1251,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1265,18 +1261,14 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Melee, Breaching (6+), Unwieldy (3)</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
+          <t>Melee, Shred</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
+          <t>2022 - Horus Heresy</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
@@ -1284,7 +1276,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Crux Malifica</t>
+          <t>Corposant Stave</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1299,36 +1291,36 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Melee, Concussive (2), Unwieldy (2)</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
+          <t>Melee, Haywire, Two-handed</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Word Bearers</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia, 2022 - Legiones Astartes, 2022 - Mechanicum, 2022 - Titan Legions</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Cthonic power claw</t>
+          <t>Crushing fists</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1343,17 +1335,17 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>User</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Specialist Weapon, Shred, Master-crafted</t>
+          <t>Melee, Breaching (6+), Unwieldy (3)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1364,7 +1356,7 @@
       <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Sons of Horus</t>
+          <t>2022 - Legiones Astartes</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
@@ -1372,7 +1364,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Decapitation Strike</t>
+          <t>Crux Malifica</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1387,17 +1379,17 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
+          <t>+3</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (3), Fleshbane, Murderous Strike (2+)</t>
+          <t>Melee, Concussive (2), Unwieldy (2)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1408,7 +1400,7 @@
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Assassins</t>
+          <t>2022 - LA - Word Bearers</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr"/>
@@ -1416,7 +1408,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Defiant</t>
+          <t>Cthonic power claw</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1431,7 +1423,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>x2</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1441,7 +1433,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Brutal (2), Specialist Weapon, Sunder</t>
+          <t>Melee, Unwieldy (2), Specialist Weapon, Shred, Master-crafted</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1452,7 +1444,7 @@
       <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Death Guard</t>
+          <t>2022 - LA - Sons of Horus</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
@@ -1460,7 +1452,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Dread saw</t>
+          <t>Decapitation Strike</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1475,17 +1467,17 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Melee, Armourbane (Melee), Unwieldy (3)</t>
+          <t>Melee, Unwieldy (3), Fleshbane, Murderous Strike (2+)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1496,7 +1488,7 @@
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Orks</t>
+          <t>2022 - LI - Assassins</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr"/>
@@ -1504,7 +1496,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Escaton Power Claw</t>
+          <t>Defiant</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1519,7 +1511,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1529,7 +1521,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Melee, Shred, Murderous Strike (6+), Unwieldy, Specialist Weapon</t>
+          <t>Melee, Unwieldy (2), Brutal (2), Specialist Weapon, Sunder</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1540,19 +1532,15 @@
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - Night Lords</t>
-        </is>
-      </c>
+          <t>2022 - LA - Death Guard</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Eviscerator</t>
+          <t>Dread saw</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1577,7 +1565,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Melee, Two-handed, Unwieldy (2)</t>
+          <t>Melee, Armourbane (Melee), Unwieldy (3)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1588,59 +1576,63 @@
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Astra Militarum</t>
+          <t>Homebrew - Orks</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Excoriator Chainaxe</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>+2</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Melee, Two-handed, Shred, Murderous Strike (5+), Unwieldy (2), Breaching (5+)</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Escaton Power Claw</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Shred, Murderous Strike (6+), Unwieldy, Specialist Weapon</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Unwieldy</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr"/>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>Master list (Exotic and Miscellaneous Melee Weapons)</t>
-        </is>
-      </c>
-      <c r="J25" s="7" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Legiones Astartes</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - Night Lords</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Excoriator Chainaxe</t>
+          <t>Eviscerator</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1655,17 +1647,17 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>x2</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Melee, Two-handed, Shred, Murderous Strike (5+), Unwieldy (2), Breaching (5+)</t>
+          <t>Melee, Two-handed, Unwieldy (2)</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -1676,63 +1668,59 @@
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, 2022 - Legiones Astartes</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - World Eaters</t>
-        </is>
-      </c>
+          <t>Homebrew - Astra Militarum</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Extricator</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Melee, Armourbane (melee), Master-crafted, Unwieldy (3)</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Excoriator Chainaxe</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Melee, Two-handed, Shred, Murderous Strike (5+), Unwieldy (2), Breaching (5+)</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Unwieldy</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - Iron Warriors</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr"/>
+      <c r="H27" s="7" t="inlineStr"/>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Exotic and Miscellaneous Melee Weapons)</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Fleshripper</t>
+          <t>Excoriator Chainaxe</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1747,17 +1735,17 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (3), Shred</t>
+          <t>Melee, Two-handed, Shred, Murderous Strike (5+), Unwieldy (2), Breaching (5+)</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -1768,15 +1756,19 @@
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
+          <t>2022 - Horus Heresy, 2022 - Legiones Astartes</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
           <t>2022 - LA - World Eaters</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Force Axe</t>
+          <t>Extricator</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1791,7 +1783,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1801,7 +1793,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Melee, Force, Unwieldy (2)</t>
+          <t>Melee, Armourbane (melee), Master-crafted, Unwieldy (3)</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -1812,19 +1804,15 @@
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes</t>
-        </is>
-      </c>
+          <t>2022 - LA - Iron Warriors</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Force Staff</t>
+          <t>Fleshripper</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1844,31 +1832,31 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Melee, Force, Reach (1)</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr"/>
+          <t>Melee, Unwieldy (3), Shred</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, Homebrew - Astra Militarum</t>
-        </is>
-      </c>
+          <t>2022 - LA - World Eaters</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Force Sword</t>
+          <t>Force Axe</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1883,20 +1871,24 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Melee, Force, Rending (6+)</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr"/>
+          <t>Melee, Force, Unwieldy (2)</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
@@ -1912,7 +1904,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Forgebreaker Desecrated</t>
+          <t>Force Staff</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1927,36 +1919,36 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (3), Master-crafted, Exoshock (3+), Brutal (2)</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
+          <t>Melee, Force, Reach (1)</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Iron Warriors</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, Homebrew - Astra Militarum</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Frost Axe</t>
+          <t>Force Sword</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1971,40 +1963,36 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>User</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Melee, Specialist weapon, Unwieldy (1), Reaping blow (1)</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
+          <t>Melee, Force, Rending (6+)</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr"/>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Space Wolves</t>
+          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Ghost Axe</t>
+          <t>Forgebreaker Desecrated</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -2019,17 +2007,17 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Melee, Brutal (2), Specialist Weapon, Unwieldy (2)</t>
+          <t>Melee, Unwieldy (3), Master-crafted, Exoshock (3+), Brutal (2)</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -2040,107 +2028,103 @@
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Asuryani)</t>
+          <t>2022 - LA - Iron Warriors</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>Graviton Crusher</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>x2</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Frost Axe</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Melee, Unwieldy (2), Haywire, Two-handed</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Specialist weapon, Unwieldy (1), Reaping blow (1)</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Unwieldy</t>
         </is>
       </c>
-      <c r="H35" s="7" t="inlineStr"/>
-      <c r="I35" s="7" t="inlineStr">
-        <is>
-          <t>Master list (Graviton Melee Weapons)</t>
-        </is>
-      </c>
-      <c r="J35" s="7" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr"/>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Legiones Astartes</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - Space Wolves</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>Graviton Crusher</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>x2</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Melee, Unwieldy (2), Haywire, Two-handed</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Horus Heresy, 2022 - Legiones Astartes</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - Iron Warriors</t>
-        </is>
-      </c>
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Gem Extractor</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Melee, Rending (6+)</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr"/>
+      <c r="H36" s="7" t="inlineStr"/>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Power Pack Weapons)</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Graviton Gauntlet</t>
+          <t>Gem Extractor</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -2155,40 +2139,32 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Specialist Weapon, Haywire</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
+          <t>Melee, Rending (6+)</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="inlineStr">
-        <is>
-          <t>2022 - BG - Blackshields, 2022 - LA - Iron Warriors</t>
-        </is>
-      </c>
+          <t>2022 - Horus Heresy</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Guardian Axe (Melee)</t>
+          <t>Ghost Axe</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -2213,7 +2189,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Melee, Two-handed, Unwieldy (2)</t>
+          <t>Melee, Brutal (2), Specialist Weapon, Unwieldy (2)</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -2224,99 +2200,107 @@
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Custodes, Homebrew - Traders Militant</t>
+          <t>Homebrew - Aeldari (Asuryani)</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>Heavy chainaxe</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>+2</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>Melee, Brutal (2), Shred, Unwieldy (2)</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Graviton Crusher</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Melee, Unwieldy (2), Haywire, Two-handed</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>Unwieldy</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Legiones Astartes</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr"/>
+      <c r="H39" s="7" t="inlineStr"/>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Graviton Melee Weapons)</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>Heavy Chainsword</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>+2</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>Melee, Shred, Two-handed, Rupture (6+)</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr"/>
-      <c r="H40" s="7" t="inlineStr"/>
-      <c r="I40" s="7" t="inlineStr">
-        <is>
-          <t>Master list (Chain Weapons)</t>
-        </is>
-      </c>
-      <c r="J40" s="7" t="inlineStr"/>
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Graviton Crusher</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Unwieldy (2), Haywire, Two-handed</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Horus Heresy, 2022 - Legiones Astartes</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - Iron Warriors</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Heavy Chainsword</t>
+          <t>Graviton Gauntlet</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -2331,36 +2315,40 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Melee, Shred, Two-handed, Rupture (6+)</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr"/>
+          <t>Melee, Unwieldy (2), Specialist Weapon, Haywire</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+          <t>2022 - Legiones Astartes</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Blood Angels, 2022 - LA - Space Wolves, 2022 - LA - Word Bearers, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes</t>
+          <t>2022 - BG - Blackshields, 2022 - LA - Iron Warriors</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Heavy Lascutter (Melee)</t>
+          <t>Guardian Axe (Melee)</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -2375,17 +2363,17 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Melee, Armourbane (Melee), Specialist Weapon, Unwieldy (4)</t>
+          <t>Melee, Two-handed, Unwieldy (2)</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -2396,7 +2384,7 @@
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia</t>
+          <t>2022 - LI - Custodes, Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr"/>
@@ -2404,7 +2392,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Helbrute hammer</t>
+          <t>Heavy chainaxe</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -2419,17 +2407,17 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Melee, Brutal (3), Unwieldy (3)</t>
+          <t>Melee, Brutal (2), Shred, Unwieldy (2)</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -2448,7 +2436,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Hellcrusher Claws</t>
+          <t>Heavy Chainsword</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
@@ -2463,24 +2451,24 @@
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>Melee, Brutal (3), Sunder</t>
+          <t>Melee, Shred, Two-handed, Rupture (6+)</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr"/>
       <c r="H44" s="7" t="inlineStr"/>
       <c r="I44" s="7" t="inlineStr">
         <is>
-          <t>Master list (Exotic and Miscellaneous Melee Weapons)</t>
+          <t>Master list (Chain Weapons)</t>
         </is>
       </c>
       <c r="J44" s="7" t="inlineStr"/>
@@ -2488,7 +2476,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Hellcrusher Claws</t>
+          <t>Heavy Chainsword</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -2503,36 +2491,36 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Melee, Brutal (3), Sunder</t>
+          <t>Melee, Shred, Two-handed, Rupture (6+)</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr"/>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, 2022 - Legiones Astartes, 2022 - Mech Library</t>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, 2022 - Mechanicum</t>
+          <t>2022 - LA - Blood Angels, 2022 - LA - Space Wolves, 2022 - LA - Word Bearers, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Indictor Axe</t>
+          <t>Heavy Lascutter (Melee)</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -2547,17 +2535,17 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Melee, Murderous Strike (6+), Rending (6+), Two-Handed, Unwieldy (1)</t>
+          <t>Melee, Armourbane (Melee), Specialist Weapon, Unwieldy (4)</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -2568,7 +2556,7 @@
       <c r="H46" s="4" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Sisters Of Silence</t>
+          <t>2022 - LI - Solar Auxilia</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr"/>
@@ -2576,7 +2564,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Killsaw</t>
+          <t>Helbrute hammer</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -2596,12 +2584,12 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Melee, Armourbane (Melee), Unwieldy (2)</t>
+          <t>Melee, Brutal (3), Unwieldy (3)</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -2612,59 +2600,55 @@
       <c r="H47" s="4" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Orks</t>
+          <t>2022 - Legiones Astartes</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>Lightning Claw</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>Melee, Rending (6+), Shred, Specialist Weapon</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr"/>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - Blood Angels, 2022 - LA - Emperor's Children, 2022 - LA - Iron Hands, 2022 - LA - Night Lords, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Thousand Sons, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LA - World Eaters, 2022 - LI - Sisters Of Silence, 2022 - Legiones Astartes</t>
-        </is>
-      </c>
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Hellcrusher Claws</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Melee, Brutal (3), Sunder</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr"/>
+      <c r="H48" s="7" t="inlineStr"/>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Exotic and Miscellaneous Melee Weapons)</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Machinator Array</t>
+          <t>Hellcrusher Claws</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2679,7 +2663,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -2689,30 +2673,26 @@
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Melee, Armourbane (Melee), Shred, Unwieldy (4)</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
+          <t>Melee, Brutal (3), Sunder</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr"/>
       <c r="H49" s="4" t="inlineStr"/>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, 2022 - Legiones Astartes, Homebrew - Traders Militant</t>
+          <t>2022 - Horus Heresy, 2022 - Legiones Astartes, 2022 - Mech Library</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Sisters Of Silence, 2022 - Mech Library, 2022 - Mechanicum</t>
+          <t>2022 - Imperialis Militia, 2022 - LI - Solar Auxilia, 2022 - Mechanicum</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Manipulator Array</t>
+          <t>Indictor Axe</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2727,7 +2707,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
@@ -2737,7 +2717,7 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (4), Shred, Armourbane (Melee), Precision Strikes (3+)</t>
+          <t>Melee, Murderous Strike (6+), Rending (6+), Two-Handed, Unwieldy (1)</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -2748,7 +2728,7 @@
       <c r="H50" s="4" t="inlineStr"/>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Iron Hands</t>
+          <t>2022 - LI - Sisters Of Silence</t>
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr"/>
@@ -2756,7 +2736,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Manos Ruinus (Cybertheurgic Weapon)</t>
+          <t>Killsaw</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2771,17 +2751,17 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>x2</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Melee, Data-djinn, Armourbane, Exoshock (3+), Unwieldy (3), Cumbersome, Cybertheurgic Focus</t>
+          <t>Melee, Armourbane (Melee), Unwieldy (2)</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -2792,63 +2772,59 @@
       <c r="H51" s="4" t="inlineStr"/>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>2022 - Mech Library</t>
-        </is>
-      </c>
-      <c r="J51" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Mechanicum</t>
-        </is>
-      </c>
+          <t>Homebrew - Orks</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>Massive crushing claws</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>x2</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Kinfolk Arc Welder</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>Melee, Unwieldy (3), Brutal (2)</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>Melee, Unwieldy (3)</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>Unwieldy</t>
         </is>
       </c>
-      <c r="H52" s="4" t="inlineStr"/>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>Homebrew - Tyranids</t>
-        </is>
-      </c>
-      <c r="J52" s="4" t="inlineStr"/>
+      <c r="H52" s="7" t="inlineStr"/>
+      <c r="I52" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Power Pack Weapons)</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Master-crafted Power Axe</t>
+          <t>Kinfolk Arc Welder</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -2863,7 +2839,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -2873,7 +2849,7 @@
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (1), Master-crafted</t>
+          <t>Melee, Unwieldy (3)</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -2884,7 +2860,7 @@
       <c r="H53" s="4" t="inlineStr"/>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>2022 - Mechanicum</t>
+          <t>2022 - Horus Heresy</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr"/>
@@ -2892,7 +2868,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Master-crafted Thunder Hammer</t>
+          <t>Lightning Claw</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -2907,36 +2883,36 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>User</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Melee, Brutal (2), Unwieldy (2), Thunderous Charge, Master-crafted</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
+          <t>Melee, Rending (6+), Shred, Specialist Weapon</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr"/>
       <c r="H54" s="4" t="inlineStr"/>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Emperor's Children</t>
-        </is>
-      </c>
-      <c r="J54" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - Blood Angels, 2022 - LA - Emperor's Children, 2022 - LA - Iron Hands, 2022 - LA - Night Lords, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Thousand Sons, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LA - World Eaters, 2022 - LI - Sisters Of Silence, 2022 - Legiones Astartes</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Melta Bomb</t>
+          <t>Machinator Array</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -2951,17 +2927,17 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>Melee, Armourbane (Melee), Detonation, Instant Death, Unwieldy (4)</t>
+          <t>Melee, Armourbane (Melee), Shred, Unwieldy (4)</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -2972,63 +2948,63 @@
       <c r="H55" s="4" t="inlineStr"/>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Asuryani)</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, 2022 - Legiones Astartes, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LI - Sisters Of Silence, 2022 - Mech Library, 2022 - Mechanicum</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>Melta Lance</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>Melee, Ungainly, Lance, Sudden Strike (2), Two-handed, One Use</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H56" s="7" t="inlineStr">
-        <is>
-          <t>2 different profiles; differs from master list</t>
-        </is>
-      </c>
-      <c r="I56" s="7" t="inlineStr">
-        <is>
-          <t>Master list (Exotic and Miscellaneous Melee Weapons)</t>
-        </is>
-      </c>
-      <c r="J56" s="7" t="inlineStr"/>
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Manipulator Array</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Unwieldy (4), Shred, Armourbane (Melee), Precision Strikes (3+)</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr"/>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - Iron Hands</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Melta Lance</t>
+          <t>Manos Ruinus (Cybertheurgic Weapon)</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -3043,7 +3019,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
@@ -3053,34 +3029,30 @@
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Melee, Ungainly, Lance, Sudden Strike (2), Two-handed, One Use</t>
+          <t>Melee, Data-djinn, Armourbane, Exoshock (3+), Unwieldy (3), Cumbersome, Cybertheurgic Focus</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H57" s="5" t="inlineStr">
-        <is>
-          <t>2 different profiles; differs from master list</t>
-        </is>
-      </c>
+          <t>Unwieldy</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr"/>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy</t>
+          <t>2022 - Mech Library</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia</t>
+          <t>2022 - Mechanicum</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Meltabombs</t>
+          <t>Massive crushing claws</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -3095,17 +3067,17 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>x2</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Melee, Armourbane (Melee), Detonation, Instant Death, Unwieldy (4)</t>
+          <t>Melee, Unwieldy (3), Brutal (2)</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -3116,19 +3088,15 @@
       <c r="H58" s="4" t="inlineStr"/>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy</t>
-        </is>
-      </c>
-      <c r="J58" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia, 2022 - LA - Alpha Legion, 2022 - LA - Blood Angels, 2022 - LA - Dark Angels, 2022 - LA - Death Guard, 2022 - LA - Emperor's Children, 2022 - LA - Imperial Fists, 2022 - LA - Iron Hands, 2022 - LA - Iron Warriors, 2022 - LA - Night Lords, 2022 - LA - Raven Guard, 2022 - LA - Salamanders, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Thousand Sons, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LA - Word Bearers, 2022 - LA - World Eaters, 2022 - LI - Assassins, 2022 - LI - Custodes, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mech Library, 2022 - Mechanicum, Homebrew - Traders Militant</t>
-        </is>
-      </c>
+          <t>Homebrew - Tyranids</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Militia Lance</t>
+          <t>Master-crafted Power Axe</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -3143,36 +3111,36 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Melee, Ungainly, Brutal (2), Sudden Strike (2), Two-handed</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr"/>
+          <t>Melee, Unwieldy (1), Master-crafted</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
       <c r="H59" s="4" t="inlineStr"/>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy</t>
-        </is>
-      </c>
-      <c r="J59" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia</t>
-        </is>
-      </c>
+          <t>2022 - Mechanicum</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Monstrous crushing claws</t>
+          <t>Master-crafted Thunder Hammer</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -3197,7 +3165,7 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (3), Brutal (2)</t>
+          <t>Melee, Brutal (2), Unwieldy (2), Thunderous Charge, Master-crafted</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -3208,7 +3176,7 @@
       <c r="H60" s="4" t="inlineStr"/>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Tyranids</t>
+          <t>2022 - LA - Emperor's Children</t>
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr"/>
@@ -3216,7 +3184,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Moz's klaw</t>
+          <t>Melta Bomb</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -3231,17 +3199,17 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2)</t>
+          <t>Melee, Armourbane (Melee), Detonation, Instant Death, Unwieldy (4)</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -3252,59 +3220,63 @@
       <c r="H61" s="4" t="inlineStr"/>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Orks</t>
+          <t>Homebrew - Aeldari (Asuryani)</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>Myrmidon Axe</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>+2</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F62" s="4" t="inlineStr">
-        <is>
-          <t>Melee, Sunder, Two-handed, Unwieldy (2)</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
-      <c r="H62" s="4" t="inlineStr"/>
-      <c r="I62" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Mechanicum</t>
-        </is>
-      </c>
-      <c r="J62" s="4" t="inlineStr"/>
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Melta Lance</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>Melee, Ungainly, Lance, Sudden Strike (2), Two-handed, One Use</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>To verify</t>
+        </is>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>2 different profiles; differs from master list</t>
+        </is>
+      </c>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Exotic and Miscellaneous Melee Weapons)</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Onager gauntlet</t>
+          <t>Melta Lance</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -3319,7 +3291,7 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
@@ -3329,26 +3301,34 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Melee, Armourbane (Melee), Unwieldy (2)</t>
+          <t>Melee, Ungainly, Lance, Sudden Strike (2), Two-handed, One Use</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
-      <c r="H63" s="4" t="inlineStr"/>
+          <t>To verify</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>2 different profiles; differs from master list</t>
+        </is>
+      </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - T'au Empire</t>
-        </is>
-      </c>
-      <c r="J63" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Power Axe</t>
+          <t>Meltabombs</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -3363,17 +3343,17 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (1)</t>
+          <t>Melee, Armourbane (Melee), Detonation, Instant Death, Unwieldy (4)</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -3384,19 +3364,19 @@
       <c r="H64" s="4" t="inlineStr"/>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Aeldari (Asuryani)</t>
+          <t>2022 - Horus Heresy</t>
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia, 2022 - LA - Alpha Legion, 2022 - LA - Blood Angels, 2022 - LA - Death Guard, 2022 - LA - Emperor's Children, 2022 - LA - Imperial Fists, 2022 - LA - Iron Hands, 2022 - LA - Night Lords, 2022 - LA - Raven Guard, 2022 - LA - Salamanders, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LA - Word Bearers, 2022 - LA - World Eaters, 2022 - LI - Custodes, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum, 2022 - Titan Legions</t>
+          <t>2022 - Imperialis Militia, 2022 - LA - Alpha Legion, 2022 - LA - Blood Angels, 2022 - LA - Dark Angels, 2022 - LA - Death Guard, 2022 - LA - Emperor's Children, 2022 - LA - Imperial Fists, 2022 - LA - Iron Hands, 2022 - LA - Iron Warriors, 2022 - LA - Night Lords, 2022 - LA - Raven Guard, 2022 - LA - Salamanders, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Thousand Sons, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LA - Word Bearers, 2022 - LA - World Eaters, 2022 - LI - Assassins, 2022 - LI - Custodes, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mech Library, 2022 - Mechanicum, Homebrew - Traders Militant</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Power Fist</t>
+          <t>Militia Lance</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -3411,40 +3391,36 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Specialist Weapon</t>
-        </is>
-      </c>
-      <c r="G65" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
+          <t>Melee, Ungainly, Brutal (2), Sudden Strike (2), Two-handed</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr"/>
       <c r="H65" s="4" t="inlineStr"/>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, 2022 - LA - Iron Warriors</t>
+          <t>2022 - Horus Heresy</t>
         </is>
       </c>
       <c r="J65" s="4" t="inlineStr">
         <is>
-          <t>2022 - Imperialis Militia, 2022 - LA - Alpha Legion, 2022 - LA - Blood Angels, 2022 - LA - Dark Angels, 2022 - LA - Death Guard, 2022 - LA - Emperor's Children, 2022 - LA - Imperial Fists, 2022 - LA - Iron Hands, 2022 - LA - Night Lords, 2022 - LA - Raven Guard, 2022 - LA - Salamanders, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Thousand Sons, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LA - Word Bearers, 2022 - LA - World Eaters, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum, 2022 - Titan Legions, Homebrew - Astra Militarum, Homebrew - Traders Militant</t>
+          <t>2022 - Imperialis Militia</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Power klaw</t>
+          <t>Monstrous crushing claws</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -3469,7 +3445,7 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Specialist Weapon</t>
+          <t>Melee, Unwieldy (3), Brutal (2)</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -3480,7 +3456,7 @@
       <c r="H66" s="4" t="inlineStr"/>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Orks</t>
+          <t>Homebrew - Tyranids</t>
         </is>
       </c>
       <c r="J66" s="4" t="inlineStr"/>
@@ -3488,7 +3464,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Power Lance</t>
+          <t>Moz's klaw</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -3503,36 +3479,36 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>x2</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Melee, Reach (1)</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr"/>
+          <t>Melee, Unwieldy (2)</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
       <c r="H67" s="4" t="inlineStr"/>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy</t>
-        </is>
-      </c>
-      <c r="J67" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia, 2022 - LA - Alpha Legion, 2022 - LA - Blood Angels, 2022 - LA - Death Guard, 2022 - LA - Emperor's Children, 2022 - LA - Imperial Fists, 2022 - LA - Iron Hands, 2022 - LA - Night Lords, 2022 - LA - Salamanders, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LI - Custodes, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum, 2022 - Titan Legions</t>
-        </is>
-      </c>
+          <t>Homebrew - Orks</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Rending claws</t>
+          <t>Myrmidon Axe</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -3547,24 +3523,28 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Melee, Rending (5+), Shred</t>
-        </is>
-      </c>
-      <c r="G68" s="3" t="inlineStr"/>
+          <t>Melee, Sunder, Two-handed, Unwieldy (2)</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
       <c r="H68" s="4" t="inlineStr"/>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes, Homebrew - Aeldari (Drukhari)</t>
+          <t>2022 - Mechanicum</t>
         </is>
       </c>
       <c r="J68" s="4" t="inlineStr"/>
@@ -3572,7 +3552,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Rime-shard</t>
+          <t>Onager gauntlet</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -3587,17 +3567,17 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>x2</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (1), Master-crafted</t>
+          <t>Melee, Armourbane (Melee), Unwieldy (2)</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -3608,63 +3588,63 @@
       <c r="H69" s="4" t="inlineStr"/>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Alpha Legion</t>
+          <t>Homebrew - T'au Empire</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="inlineStr">
-        <is>
-          <t>Ripper Gun</t>
-        </is>
-      </c>
-      <c r="B70" s="6" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C70" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D70" s="6" t="inlineStr">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Power Axe</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
       </c>
-      <c r="E70" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F70" s="7" t="inlineStr">
-        <is>
-          <t>Melee, Reaping Blow (1), Two-handed</t>
-        </is>
-      </c>
-      <c r="G70" s="6" t="inlineStr">
-        <is>
-          <t>To verify</t>
-        </is>
-      </c>
-      <c r="H70" s="7" t="inlineStr">
-        <is>
-          <t>differs from master list</t>
-        </is>
-      </c>
-      <c r="I70" s="7" t="inlineStr">
-        <is>
-          <t>Master list (Exotic and Miscellaneous Melee Weapons)</t>
-        </is>
-      </c>
-      <c r="J70" s="7" t="inlineStr"/>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Unwieldy (1)</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr"/>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Horus Heresy, Homebrew - Aeldari (Asuryani)</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia, 2022 - LA - Alpha Legion, 2022 - LA - Blood Angels, 2022 - LA - Death Guard, 2022 - LA - Emperor's Children, 2022 - LA - Imperial Fists, 2022 - LA - Iron Hands, 2022 - LA - Night Lords, 2022 - LA - Raven Guard, 2022 - LA - Salamanders, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LA - Word Bearers, 2022 - LA - World Eaters, 2022 - LI - Custodes, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum, 2022 - Titan Legions</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Saturnine Disruption Fist</t>
+          <t>Power Fist</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -3689,7 +3669,7 @@
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>Melee, Brutal (2), Unwieldy (3), Specialist Weapon</t>
+          <t>Melee, Unwieldy (2), Specialist Weapon</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -3700,15 +3680,19 @@
       <c r="H71" s="4" t="inlineStr"/>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
-        </is>
-      </c>
-      <c r="J71" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, 2022 - LA - Iron Warriors</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia, 2022 - LA - Alpha Legion, 2022 - LA - Blood Angels, 2022 - LA - Dark Angels, 2022 - LA - Death Guard, 2022 - LA - Emperor's Children, 2022 - LA - Imperial Fists, 2022 - LA - Iron Hands, 2022 - LA - Night Lords, 2022 - LA - Raven Guard, 2022 - LA - Salamanders, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Thousand Sons, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LA - Word Bearers, 2022 - LA - World Eaters, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum, 2022 - Titan Legions, Homebrew - Astra Militarum, Homebrew - Traders Militant</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Servo-Arm</t>
+          <t>Power klaw</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -3723,7 +3707,7 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>x2</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
@@ -3733,7 +3717,7 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Melee, Extra Attacks (1), Unwieldy (3)</t>
+          <t>Melee, Unwieldy (2), Specialist Weapon</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -3744,19 +3728,15 @@
       <c r="H72" s="4" t="inlineStr"/>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J72" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia, 2022 - LA - Iron Hands, 2022 - LA - Iron Warriors, 2022 - LA - Thousand Sons, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum</t>
-        </is>
-      </c>
+          <t>Homebrew - Orks</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Singing spear (melee)</t>
+          <t>Power Lance</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -3771,32 +3751,36 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>Melee, Force, Murderous Strike (6+)</t>
+          <t>Melee, Reach (1)</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr"/>
       <c r="H73" s="4" t="inlineStr"/>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani)</t>
-        </is>
-      </c>
-      <c r="J73" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia, 2022 - LA - Alpha Legion, 2022 - LA - Blood Angels, 2022 - LA - Death Guard, 2022 - LA - Emperor's Children, 2022 - LA - Imperial Fists, 2022 - LA - Iron Hands, 2022 - LA - Night Lords, 2022 - LA - Salamanders, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LI - Custodes, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum, 2022 - Titan Legions</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Solarite Power Gauntlet</t>
+          <t>Rending claws</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -3811,40 +3795,32 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>User</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2)</t>
-        </is>
-      </c>
-      <c r="G74" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
+          <t>Melee, Rending (5+), Shred</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr"/>
       <c r="H74" s="4" t="inlineStr"/>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Custodes, 2022 - Legiones Astartes, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J74" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - Imperial Fists</t>
-        </is>
-      </c>
+          <t>2022 - Legiones Astartes, Homebrew - Aeldari (Drukhari)</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Sovereign Greatblade</t>
+          <t>Rime-shard</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -3859,17 +3835,17 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Melee, Brutal (3), Murderous Strike (5+), Unwieldy (3)</t>
+          <t>Melee, Unwieldy (1), Master-crafted</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -3880,59 +3856,63 @@
       <c r="H75" s="4" t="inlineStr"/>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>2022 - Daemons - Daemons of the Ruinstorm</t>
+          <t>2022 - LA - Alpha Legion</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="3" t="inlineStr">
-        <is>
-          <t>Split the Mountain</t>
-        </is>
-      </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>Melee</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>+3</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>Melee, Unwieldy (2), Master-crafted</t>
-        </is>
-      </c>
-      <c r="G76" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
-      <c r="H76" s="4" t="inlineStr"/>
-      <c r="I76" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - White Scars</t>
-        </is>
-      </c>
-      <c r="J76" s="4" t="inlineStr"/>
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Ripper Gun</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>Melee, Reaping Blow (1), Two-handed</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>To verify</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>differs from master list</t>
+        </is>
+      </c>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Exotic and Miscellaneous Melee Weapons)</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Staff of Dark Authority</t>
+          <t>Saturnine Disruption Fist</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -3947,17 +3927,17 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>x2</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Murderous Strike (6+)</t>
+          <t>Melee, Brutal (2), Unwieldy (3), Specialist Weapon</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -3976,7 +3956,7 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Storm Axe</t>
+          <t>Servo-Arm</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -3991,7 +3971,7 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
@@ -4001,7 +3981,7 @@
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Two-handed, Murderous Strike (6+)</t>
+          <t>Melee, Extra Attacks (1), Unwieldy (3)</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -4012,15 +3992,19 @@
       <c r="H78" s="4" t="inlineStr"/>
       <c r="I78" s="4" t="inlineStr">
         <is>
-          <t>2022 - LI - Solar Auxilia, Homebrew - Traders Militant</t>
-        </is>
-      </c>
-      <c r="J78" s="4" t="inlineStr"/>
+          <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia, 2022 - LA - Iron Hands, 2022 - LA - Iron Warriors, 2022 - LA - Thousand Sons, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, 2022 - Mechanicum</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Subjugator</t>
+          <t>Singing spear (melee)</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -4035,28 +4019,24 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>User</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Brutal (2), Reaping Blow (1)</t>
-        </is>
-      </c>
-      <c r="G79" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
+          <t>Melee, Force, Murderous Strike (6+)</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr"/>
       <c r="H79" s="4" t="inlineStr"/>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Imperial Fists</t>
+          <t>Homebrew - Aeldari (Anhrathe), Homebrew - Aeldari (Asuryani)</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr"/>
@@ -4064,7 +4044,7 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Sundering Blows</t>
+          <t>Solarite Power Gauntlet</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -4079,7 +4059,7 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
@@ -4089,7 +4069,7 @@
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Melee, Brutal (2), Wrathful Blows (3), Unwieldy (3)</t>
+          <t>Melee, Unwieldy (2)</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -4100,15 +4080,19 @@
       <c r="H80" s="4" t="inlineStr"/>
       <c r="I80" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Emperor's Children</t>
-        </is>
-      </c>
-      <c r="J80" s="4" t="inlineStr"/>
+          <t>2022 - LI - Custodes, 2022 - Legiones Astartes, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - Imperial Fists</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Tactus Mors (Cybertheurgic Weapon)</t>
+          <t>Sovereign Greatblade</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -4123,17 +4107,17 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (3), Haywire, Cybertheurgic Focus</t>
+          <t>Melee, Brutal (3), Murderous Strike (5+), Unwieldy (3)</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -4144,7 +4128,7 @@
       <c r="H81" s="4" t="inlineStr"/>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>2022 - Mech Library</t>
+          <t>2022 - Daemons - Daemons of the Ruinstorm</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr"/>
@@ -4152,7 +4136,7 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Tainted Axe</t>
+          <t>Split the Mountain</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -4167,7 +4151,7 @@
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
@@ -4177,7 +4161,7 @@
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (1), Murderous Strike (6+)</t>
+          <t>Melee, Unwieldy (2), Master-crafted</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -4188,7 +4172,7 @@
       <c r="H82" s="4" t="inlineStr"/>
       <c r="I82" s="4" t="inlineStr">
         <is>
-          <t>2022 - Legiones Astartes</t>
+          <t>2022 - LA - White Scars</t>
         </is>
       </c>
       <c r="J82" s="4" t="inlineStr"/>
@@ -4196,7 +4180,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Tankhammer</t>
+          <t>Staff of Dark Authority</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -4211,17 +4195,17 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Melee, Armourbane (Melee), Unwieldy (2), Two-Handed, Gets Hot</t>
+          <t>Melee, Unwieldy (2), Murderous Strike (6+)</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -4232,7 +4216,7 @@
       <c r="H83" s="4" t="inlineStr"/>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Orks</t>
+          <t>2022 - Legiones Astartes</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr"/>
@@ -4240,7 +4224,7 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Terrawat-pattern Power Gauntlet</t>
+          <t>Storm Axe</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -4255,7 +4239,7 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
@@ -4265,7 +4249,7 @@
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Specialist Weapon, Brutal (2), Charged Attacks</t>
+          <t>Melee, Unwieldy (2), Two-handed, Murderous Strike (6+)</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -4276,7 +4260,7 @@
       <c r="H84" s="4" t="inlineStr"/>
       <c r="I84" s="4" t="inlineStr">
         <is>
-          <t>2022 - BG - Blackshields</t>
+          <t>2022 - LI - Solar Auxilia, Homebrew - Traders Militant</t>
         </is>
       </c>
       <c r="J84" s="4" t="inlineStr"/>
@@ -4284,7 +4268,7 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>The Axe of Castigation (Overhead Strike)</t>
+          <t>Subjugator</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -4299,17 +4283,17 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>Melee, Two-handed, Unwieldy (2), Master-crafted</t>
+          <t>Melee, Unwieldy (2), Brutal (2), Reaping Blow (1)</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -4320,7 +4304,7 @@
       <c r="H85" s="4" t="inlineStr"/>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Dark Angels</t>
+          <t>2022 - LA - Imperial Fists</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr"/>
@@ -4328,7 +4312,7 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>The Azurda Char'is</t>
+          <t>Sundering Blows</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -4343,17 +4327,17 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Force</t>
+          <t>Melee, Brutal (2), Wrathful Blows (3), Unwieldy (3)</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
@@ -4364,7 +4348,7 @@
       <c r="H86" s="4" t="inlineStr"/>
       <c r="I86" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Word Bearers</t>
+          <t>2022 - LA - Emperor's Children</t>
         </is>
       </c>
       <c r="J86" s="4" t="inlineStr"/>
@@ -4372,7 +4356,7 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>The Death of Worlds</t>
+          <t>Tactus Mors (Cybertheurgic Weapon)</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -4387,17 +4371,17 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>+5</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Two-handed, Curse of Dead Worlds</t>
+          <t>Melee, Unwieldy (3), Haywire, Cybertheurgic Focus</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -4408,7 +4392,7 @@
       <c r="H87" s="4" t="inlineStr"/>
       <c r="I87" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Dark Angels</t>
+          <t>2022 - Mech Library</t>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr"/>
@@ -4416,7 +4400,7 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>The Hand of Dominion</t>
+          <t>Tainted Axe</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -4431,17 +4415,17 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Brutal (2), Master-crafted, Specialist Weapon</t>
+          <t>Melee, Unwieldy (1), Murderous Strike (6+)</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
@@ -4452,7 +4436,7 @@
       <c r="H88" s="4" t="inlineStr"/>
       <c r="I88" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Ultramarines</t>
+          <t>2022 - Legiones Astartes</t>
         </is>
       </c>
       <c r="J88" s="4" t="inlineStr"/>
@@ -4460,7 +4444,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>The Prophet</t>
+          <t>Tankhammer</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -4475,17 +4459,17 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (3), Thunderstrike</t>
+          <t>Melee, Armourbane (Melee), Unwieldy (2), Two-Handed, Gets Hot</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
@@ -4496,7 +4480,7 @@
       <c r="H89" s="4" t="inlineStr"/>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Alpha Legion</t>
+          <t>Homebrew - Orks</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr"/>
@@ -4504,7 +4488,7 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Thunder Hammer</t>
+          <t>Terrawat-pattern Power Gauntlet</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -4529,7 +4513,7 @@
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (3), Brutal (2), Specialist Weapon</t>
+          <t>Melee, Unwieldy (2), Specialist Weapon, Brutal (2), Charged Attacks</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -4540,19 +4524,15 @@
       <c r="H90" s="4" t="inlineStr"/>
       <c r="I90" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy</t>
-        </is>
-      </c>
-      <c r="J90" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia, 2022 - LA - Blood Angels, 2022 - LA - Dark Angels, 2022 - LA - Imperial Fists, 2022 - LA - Iron Hands, 2022 - LA - Iron Warriors, 2022 - LA - Night Lords, 2022 - LA - Salamanders, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Thousand Sons, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LA - World Eaters, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, Homebrew - Traders Militant</t>
-        </is>
-      </c>
+          <t>2022 - BG - Blackshields</t>
+        </is>
+      </c>
+      <c r="J90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Tians'han</t>
+          <t>The Axe of Castigation (Overhead Strike)</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -4567,7 +4547,7 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
@@ -4577,7 +4557,7 @@
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (3), Brutal (2), Specialist Weapon, Reaping Blow (1), Hammerhand</t>
+          <t>Melee, Two-handed, Unwieldy (2), Master-crafted</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
@@ -4588,7 +4568,7 @@
       <c r="H91" s="4" t="inlineStr"/>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - White Scars</t>
+          <t>2022 - LA - Dark Angels</t>
         </is>
       </c>
       <c r="J91" s="4" t="inlineStr"/>
@@ -4596,7 +4576,7 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Voidscythe</t>
+          <t>The Azurda Char'is</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -4611,17 +4591,17 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>User</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Melee, Unwieldy (2), Rending (5+), Armourbane (Melee)</t>
+          <t>Melee, Unwieldy (2), Force</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr">
@@ -4632,7 +4612,7 @@
       <c r="H92" s="4" t="inlineStr"/>
       <c r="I92" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Necrons</t>
+          <t>2022 - LA - Word Bearers</t>
         </is>
       </c>
       <c r="J92" s="4" t="inlineStr"/>
@@ -4640,7 +4620,7 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Worldbreaker</t>
+          <t>The Death of Worlds</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -4655,7 +4635,7 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
@@ -4665,7 +4645,7 @@
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Melee, Master-crafted, Brutal (2), Sunder, Unwieldy (3)</t>
+          <t>Melee, Unwieldy (2), Two-handed, Curse of Dead Worlds</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
@@ -4676,7 +4656,7 @@
       <c r="H93" s="4" t="inlineStr"/>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>2022 - LA - Sons of Horus</t>
+          <t>2022 - LA - Dark Angels</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr"/>
@@ -4684,7 +4664,7 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>Wraithsword – Piercing Blow</t>
+          <t>The Hand of Dominion</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -4709,7 +4689,7 @@
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Melee, Murderous Strike (5+), Two-Handed, Unwieldy (3)</t>
+          <t>Melee, Unwieldy (2), Brutal (2), Master-crafted, Specialist Weapon</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
@@ -4720,7 +4700,7 @@
       <c r="H94" s="4" t="inlineStr"/>
       <c r="I94" s="4" t="inlineStr">
         <is>
-          <t>Homebrew - Aeldari (Asuryani)</t>
+          <t>2022 - LA - Ultramarines</t>
         </is>
       </c>
       <c r="J94" s="4" t="inlineStr"/>
@@ -4728,7 +4708,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Wrecker claws (Stone-crusher)</t>
+          <t>The Prophet</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -4743,7 +4723,7 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>x2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
@@ -4753,7 +4733,7 @@
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Melee, Brutal (2), Armourbane (Melee), Unwieldy (3), Wrecker</t>
+          <t>Melee, Unwieldy (3), Thunderstrike</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
@@ -4764,20 +4744,288 @@
       <c r="H95" s="4" t="inlineStr"/>
       <c r="I95" s="4" t="inlineStr">
         <is>
+          <t>2022 - LA - Alpha Legion</t>
+        </is>
+      </c>
+      <c r="J95" s="4" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>Thunder Hammer</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Unwieldy (3), Brutal (2), Specialist Weapon</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr"/>
+      <c r="I96" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Horus Heresy</t>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia, 2022 - LA - Blood Angels, 2022 - LA - Dark Angels, 2022 - LA - Imperial Fists, 2022 - LA - Iron Hands, 2022 - LA - Iron Warriors, 2022 - LA - Night Lords, 2022 - LA - Salamanders, 2022 - LA - Sons of Horus, 2022 - LA - Space Wolves, 2022 - LA - Thousand Sons, 2022 - LA - Ultramarines, 2022 - LA - White Scars, 2022 - LA - World Eaters, 2022 - LI - Sisters Of Silence, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes, Homebrew - Traders Militant</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>Tians'han</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Unwieldy (3), Brutal (2), Specialist Weapon, Reaping Blow (1), Hammerhand</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr"/>
+      <c r="I97" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - White Scars</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>Voidscythe</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Unwieldy (2), Rending (5+), Armourbane (Melee)</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr"/>
+      <c r="I98" s="4" t="inlineStr">
+        <is>
+          <t>Homebrew - Necrons</t>
+        </is>
+      </c>
+      <c r="J98" s="4" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>Worldbreaker</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Master-crafted, Brutal (2), Sunder, Unwieldy (3)</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr"/>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>2022 - LA - Sons of Horus</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>Wraithsword – Piercing Blow</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Murderous Strike (5+), Two-Handed, Unwieldy (3)</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr"/>
+      <c r="I100" s="4" t="inlineStr">
+        <is>
+          <t>Homebrew - Aeldari (Asuryani)</t>
+        </is>
+      </c>
+      <c r="J100" s="4" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>Wrecker claws (Stone-crusher)</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>Melee, Brutal (2), Armourbane (Melee), Unwieldy (3), Wrecker</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr"/>
+      <c r="I101" s="4" t="inlineStr">
+        <is>
           <t>Homebrew - Tyranids</t>
         </is>
       </c>
-      <c r="J95" s="4" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="8" t="inlineStr">
+      <c r="J101" s="4" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
         <is>
           <t>Rows shaded blue are the master weapon list (homebrew/source/additional-weapons.md); other rows are catalogue/gst profiles. 'Defined in' is the file holding the profile; 'Used by' is catalogues linking to it.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J95"/>
+  <autoFilter ref="A1:J101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6794,7 +7042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -9270,93 +9518,89 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>The Devil's Due</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Stone Burner</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>Ranged</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>+2</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>6"</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>Unwieldy (3), The Devil's Due, Murderous Strike (6+), Master-crafted</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>Unwieldy</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="inlineStr"/>
-      <c r="I58" s="4" t="inlineStr">
-        <is>
-          <t>2022 - LA - Night Lords</t>
-        </is>
-      </c>
-      <c r="J58" s="4" t="inlineStr"/>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>Pistol 1, Armourbane (Melta)</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr"/>
+      <c r="H58" s="7" t="inlineStr"/>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Power Pack Weapons)</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>Thunderblast Cannon</t>
-        </is>
-      </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Stone Burner</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>Ranged</t>
         </is>
       </c>
-      <c r="C59" s="6" t="inlineStr">
-        <is>
-          <t>72"</t>
-        </is>
-      </c>
-      <c r="D59" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F59" s="7" t="inlineStr">
-        <is>
-          <t>Ordnance 1, Large Blast (5"), Rupture (5+), Pinning</t>
-        </is>
-      </c>
-      <c r="G59" s="6" t="inlineStr"/>
-      <c r="H59" s="7" t="inlineStr"/>
-      <c r="I59" s="7" t="inlineStr">
-        <is>
-          <t>Master list (Artillery Weapons)</t>
-        </is>
-      </c>
-      <c r="J59" s="7" t="inlineStr"/>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>6"</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Pistol 1, Armourbane (Melta)</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr"/>
+      <c r="H59" s="4" t="inlineStr"/>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Horus Heresy</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Thunderblast Cannon</t>
+          <t>The Devil's Due</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -9366,85 +9610,81 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>72"</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Ordnance 1, Large Blast (5"), Rupture (5+), Pinning</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="inlineStr"/>
+          <t>Unwieldy (3), The Devil's Due, Murderous Strike (6+), Master-crafted</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Unwieldy</t>
+        </is>
+      </c>
       <c r="H60" s="4" t="inlineStr"/>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>2022 - Horus Heresy</t>
-        </is>
-      </c>
-      <c r="J60" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia</t>
-        </is>
-      </c>
+          <t>2022 - LA - Night Lords</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>Thunderstub</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>Thunderblast Cannon</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>Ranged</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>6"</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>72"</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>Pistol 1, Brutal (2), Concussive (1)</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr"/>
-      <c r="H61" s="4" t="inlineStr"/>
-      <c r="I61" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Horus Heresy</t>
-        </is>
-      </c>
-      <c r="J61" s="4" t="inlineStr">
-        <is>
-          <t>2022 - Imperialis Militia</t>
-        </is>
-      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>Ordnance 1, Large Blast (5"), Rupture (5+), Pinning</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr"/>
+      <c r="H61" s="7" t="inlineStr"/>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>Master list (Artillery Weapons)</t>
+        </is>
+      </c>
+      <c r="J61" s="7" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Volkite Dual-Culverin</t>
+          <t>Thunderblast Cannon</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -9454,46 +9694,134 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>45"</t>
+          <t>72"</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Heavy 6, Deflagrate, Twin-linked</t>
+          <t>Ordnance 1, Large Blast (5"), Rupture (5+), Pinning</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr"/>
       <c r="H62" s="4" t="inlineStr"/>
       <c r="I62" s="4" t="inlineStr">
         <is>
+          <t>2022 - Horus Heresy</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Thunderstub</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Ranged</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>6"</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Pistol 1, Brutal (2), Concussive (1)</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr"/>
+      <c r="H63" s="4" t="inlineStr"/>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Horus Heresy</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>2022 - Imperialis Militia</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Volkite Dual-Culverin</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Ranged</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>45"</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>Heavy 6, Deflagrate, Twin-linked</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr"/>
+      <c r="H64" s="4" t="inlineStr"/>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
           <t>2022 - Horus Heresy, Homebrew - Traders Militant</t>
         </is>
       </c>
-      <c r="J62" s="4" t="inlineStr">
+      <c r="J64" s="4" t="inlineStr">
         <is>
           <t>2022 - LA - Thousand Sons, 2022 - LI - Custodes, 2022 - LI - Solar Auxilia, 2022 - Legiones Astartes</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>Rows shaded blue are the master weapon list (homebrew/source/additional-weapons.md); other rows are catalogue/gst profiles. 'Defined in' is the file holding the profile; 'Used by' is catalogues linking to it.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J62"/>
+  <autoFilter ref="A1:J64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>